<commit_message>
Fix: update buoyancy_estimates.xlsx and cache bust
</commit_message>
<xml_diff>
--- a/PRFS_II/buoyancy_estimates.xlsx
+++ b/PRFS_II/buoyancy_estimates.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\Pakistan_Income_Tax_Slabs_app\PRFS_II\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\Pakistan_Income_Tax_Slabs_app\macro_forecasting_II\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4848484C-A1C4-4453-B26C-4AA2DF788457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA7018C2-B8F0-4975-8E45-068EED795E10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" xr2:uid="{A220C3EB-FB50-4D70-8594-0EAD70902D49}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10276" firstSheet="1" activeTab="3" xr2:uid="{A220C3EB-FB50-4D70-8594-0EAD70902D49}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Tax &amp; Tax Base" sheetId="1" r:id="rId1"/>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>Data Sources: Federal Board of Revenue (FBR) Forecasting 2024–25; FBR Yearbook 2024–25; Budget Brief 2025–26; Ministry of Finance (MoF) Estimates, Pakistan Bureau of Statistics</t>
+  </si>
+  <si>
+    <t>Note: Total sales figures were available for 2025-26; therefore, the historical sales tax on import-to-total sales ratio (average of the past five years) was applied to estimate import sales and the same was done for domestic good sales tax</t>
   </si>
   <si>
     <t>Agriculture GDP for 2025–26 is estimated by applying the last five-year average agriculture share in GDP (23%) to total GDP. Dutiable imports are estimated by applying the last five-year average dutiable share of total imports (47%) to total imports (goods).</t>
@@ -469,9 +472,6 @@
   </si>
   <si>
     <t>[11,967, 18,438]</t>
-  </si>
-  <si>
-    <t>Note: Total sales figures were available not  2025-26; therefore, the historical sales tax on import-to-total sales ratio (average of the past five years) was applied to estimate import sales and the same was done for domestic good sales tax</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1485,7 @@
   <sheetData>
     <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="49" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O1" s="42"/>
     </row>
@@ -2981,7 +2981,7 @@
     <row r="34" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B34" s="27"/>
       <c r="C34" s="34" t="s">
-        <v>131</v>
+        <v>79</v>
       </c>
       <c r="L34" s="28"/>
       <c r="N34" s="26"/>
@@ -2991,7 +2991,7 @@
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.45">
       <c r="C35" s="44" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="2:17" x14ac:dyDescent="0.45">
@@ -3045,7 +3045,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="49" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.45">
@@ -4457,16 +4457,16 @@
     </row>
     <row r="39" spans="3:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C39" s="84" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D39" s="84"/>
       <c r="E39" s="85" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F39" s="85"/>
       <c r="G39" s="85"/>
       <c r="H39" s="84" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I39" s="84"/>
       <c r="J39" s="84"/>
@@ -4643,7 +4643,7 @@
   <sheetData>
     <row r="2" spans="1:8" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B2" s="70" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C2" s="71" t="s">
         <v>70</v>
@@ -4652,16 +4652,16 @@
         <v>71</v>
       </c>
       <c r="E2" s="71" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F2" s="70" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G2" s="70" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H2" s="71" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
@@ -4678,13 +4678,13 @@
         <v>7329</v>
       </c>
       <c r="F3" s="74" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G3" s="74" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H3" s="74" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
@@ -4698,16 +4698,16 @@
         <v>1946.8027617846731</v>
       </c>
       <c r="E4" s="73" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F4" s="75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G4" s="75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H4" s="75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.45">
@@ -4721,16 +4721,16 @@
         <v>3291.1521078734595</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F5" s="75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G5" s="75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H5" s="75" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.45">
@@ -4747,13 +4747,13 @@
         <v>4730</v>
       </c>
       <c r="F6" s="74" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G6" s="74" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H6" s="74" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
@@ -4770,13 +4770,13 @@
         <v>1592</v>
       </c>
       <c r="F7" s="74" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G7" s="74" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H7" s="74" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.45">
@@ -4793,13 +4793,13 @@
         <v>1399</v>
       </c>
       <c r="F8" s="74" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G8" s="74" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H8" s="74" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.45">
@@ -4816,10 +4816,10 @@
         <v>15051</v>
       </c>
       <c r="F9" s="74" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G9" s="74" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H9" s="74"/>
     </row>
@@ -4882,7 +4882,7 @@
   <sheetPr>
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="29.86328125" customWidth="1"/>
@@ -4895,12 +4895,12 @@
     <col min="9" max="9" width="9.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="49" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="26.25" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="26.25" x14ac:dyDescent="0.45">
       <c r="B5" s="86" t="s">
         <v>74</v>
       </c>
@@ -4926,33 +4926,31 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B6" s="86"/>
       <c r="C6" s="35">
-        <v>6902000</v>
+        <v>6755478</v>
       </c>
       <c r="D6" s="41">
-        <f>0.61*F6</f>
-        <v>2899330</v>
+        <v>2640955</v>
       </c>
       <c r="E6" s="35">
-        <f>F6*0.39</f>
-        <v>1853670</v>
+        <v>1688480</v>
       </c>
       <c r="F6" s="35">
-        <v>4753000</v>
+        <v>4329435</v>
       </c>
       <c r="G6" s="41">
-        <v>888000</v>
+        <v>839352</v>
       </c>
       <c r="H6" s="41">
-        <v>1588000</v>
+        <v>1309059</v>
       </c>
       <c r="I6" s="35">
-        <v>14131000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+        <v>13233324</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B7" s="66"/>
       <c r="C7" s="67"/>
       <c r="D7" s="68"/>
@@ -4961,8 +4959,15 @@
       <c r="G7" s="68"/>
       <c r="H7" s="68"/>
       <c r="I7" s="67"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -4974,7 +4979,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B9" s="47"/>
       <c r="C9" s="47" t="s">
         <v>42</v>
@@ -4998,106 +5003,106 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:18" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="19" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="6">
         <f>'Sensitivity Analysis'!C6/1000</f>
-        <v>6902</v>
+        <v>6755.4780000000001</v>
       </c>
       <c r="D10" s="7">
         <f>'Sensitivity Analysis'!E6/1000</f>
-        <v>1853.67</v>
+        <v>1688.48</v>
       </c>
       <c r="E10" s="7">
         <f>'Sensitivity Analysis'!D6/1000</f>
-        <v>2899.33</v>
+        <v>2640.9549999999999</v>
       </c>
       <c r="F10" s="7">
         <f>SUM(D10:E10)</f>
-        <v>4753</v>
+        <v>4329.4349999999995</v>
       </c>
       <c r="G10" s="6">
         <f>H6/1000</f>
-        <v>1588</v>
+        <v>1309.059</v>
       </c>
       <c r="H10" s="6">
         <f>G6/1000</f>
-        <v>888</v>
+        <v>839.35199999999998</v>
       </c>
       <c r="I10" s="6">
         <f>I6/1000</f>
-        <v>14131</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="29.65" customHeight="1" x14ac:dyDescent="0.45">
+        <v>13233.324000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="29.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="19" t="s">
         <v>59</v>
       </c>
       <c r="C11" s="7">
         <f>C10*('Tax Buoyancy Estimates'!J40/100)</f>
-        <v>924.18230818709912</v>
+        <v>904.56291668315964</v>
       </c>
       <c r="D11" s="8">
         <f>D10*('Tax Buoyancy Estimates'!J41/100)</f>
-        <v>93.132761784673008</v>
+        <v>84.833225772756023</v>
       </c>
       <c r="E11" s="8">
         <f>E10*('Tax Buoyancy Estimates'!J42/100)</f>
-        <v>391.82210787345952</v>
+        <v>356.90471760680992</v>
       </c>
       <c r="F11" s="8">
         <f>SUM(D11:E11)</f>
-        <v>484.95486965813251</v>
+        <v>441.73794337956593</v>
       </c>
       <c r="G11" s="7">
         <f>G10*('Tax Buoyancy Estimates'!J43/100)</f>
-        <v>220.54747001295391</v>
+        <v>181.80708472776286</v>
       </c>
       <c r="H11" s="9">
         <f>H10*('Tax Buoyancy Estimates'!J44/100)</f>
-        <v>38.290437907385439</v>
+        <v>36.192742836080839</v>
       </c>
       <c r="I11" s="8">
         <f>SUM(C11,F11,G11,H11)</f>
-        <v>1667.9750857655711</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
+        <v>1564.3006876265695</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="19" t="s">
         <v>71</v>
       </c>
       <c r="C12" s="7">
         <f t="shared" ref="C12:H12" si="0">C10+C11</f>
-        <v>7826.1823081870989</v>
+        <v>7660.0409166831596</v>
       </c>
       <c r="D12" s="7">
         <f t="shared" si="0"/>
-        <v>1946.8027617846731</v>
+        <v>1773.3132257727561</v>
       </c>
       <c r="E12" s="7">
         <f t="shared" si="0"/>
-        <v>3291.1521078734595</v>
+        <v>2997.8597176068097</v>
       </c>
       <c r="F12" s="7">
         <f>F10+F11</f>
-        <v>5237.9548696581323</v>
+        <v>4771.1729433795654</v>
       </c>
       <c r="G12" s="7">
         <f t="shared" si="0"/>
-        <v>1808.5474700129539</v>
+        <v>1490.8660847277629</v>
       </c>
       <c r="H12" s="7">
         <f t="shared" si="0"/>
-        <v>926.29043790738547</v>
+        <v>875.54474283608079</v>
       </c>
       <c r="I12" s="7">
         <f>I10+I11</f>
-        <v>15798.975085765571</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+        <v>14797.62468762657</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B13" s="19" t="s">
         <v>60</v>
       </c>
@@ -5130,7 +5135,7 @@
         <v>50.128897053868883</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -5140,7 +5145,7 @@
       <c r="H14" s="10"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -5150,7 +5155,7 @@
       <c r="H15" s="10"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -5214,31 +5219,31 @@
       </c>
       <c r="C20" s="7">
         <f t="shared" ref="C20:I20" si="1">C10</f>
-        <v>6902</v>
+        <v>6755.4780000000001</v>
       </c>
       <c r="D20" s="7">
         <f t="shared" si="1"/>
-        <v>1853.67</v>
+        <v>1688.48</v>
       </c>
       <c r="E20" s="7">
         <f t="shared" si="1"/>
-        <v>2899.33</v>
+        <v>2640.9549999999999</v>
       </c>
       <c r="F20" s="7">
         <f t="shared" si="1"/>
-        <v>4753</v>
+        <v>4329.4349999999995</v>
       </c>
       <c r="G20" s="7">
         <f t="shared" si="1"/>
-        <v>1588</v>
+        <v>1309.059</v>
       </c>
       <c r="H20" s="7">
         <f t="shared" si="1"/>
-        <v>888</v>
+        <v>839.35199999999998</v>
       </c>
       <c r="I20" s="7">
         <f t="shared" si="1"/>
-        <v>14131</v>
+        <v>13233.324000000001</v>
       </c>
     </row>
     <row r="21" spans="2:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -5280,25 +5285,25 @@
       </c>
       <c r="C22" s="7">
         <f>C20*(1+(C21/100))</f>
-        <v>7733.7640773683897</v>
+        <v>7569.5846250148443</v>
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="7"/>
       <c r="F22" s="7">
         <f>F20*(1+(F21/100))</f>
-        <v>5546.0199499090786</v>
+        <v>5051.7847426540311</v>
       </c>
       <c r="G22" s="7">
         <f>G20*(1+(G21/100))</f>
-        <v>1786.4927230116587</v>
+        <v>1472.6853762549867</v>
       </c>
       <c r="H22" s="7">
         <f>H20*(1+(H21/100))</f>
-        <v>922.46139411664694</v>
+        <v>871.92546855247281</v>
       </c>
       <c r="I22" s="7">
         <f>I20*(1+(I21/100))</f>
-        <v>20506.342998413991</v>
+        <v>19203.671428288431</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.45">
@@ -5323,7 +5328,7 @@
     </row>
     <row r="25" spans="2:9" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B25" s="48" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C25" s="47" t="s">
         <v>42</v>
@@ -5353,31 +5358,31 @@
       </c>
       <c r="C26" s="7">
         <f t="shared" ref="C26:I26" si="3">C10</f>
-        <v>6902</v>
+        <v>6755.4780000000001</v>
       </c>
       <c r="D26" s="7">
         <f t="shared" si="3"/>
-        <v>1853.67</v>
+        <v>1688.48</v>
       </c>
       <c r="E26" s="7">
         <f t="shared" si="3"/>
-        <v>2899.33</v>
+        <v>2640.9549999999999</v>
       </c>
       <c r="F26" s="7">
         <f t="shared" si="3"/>
-        <v>4753</v>
+        <v>4329.4349999999995</v>
       </c>
       <c r="G26" s="7">
         <f t="shared" si="3"/>
-        <v>1588</v>
+        <v>1309.059</v>
       </c>
       <c r="H26" s="7">
         <f t="shared" si="3"/>
-        <v>888</v>
+        <v>839.35199999999998</v>
       </c>
       <c r="I26" s="7">
         <f t="shared" si="3"/>
-        <v>14131</v>
+        <v>13233.324000000001</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -5419,25 +5424,25 @@
       </c>
       <c r="C28" s="7">
         <f>C26*(1+(C27/100))</f>
-        <v>7918.600539005809</v>
+        <v>7750.4972083514758</v>
       </c>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
       <c r="F28" s="7">
         <f>F26*(1+(F27/100))</f>
-        <v>5722.2466054444294</v>
+        <v>5212.3069076882603</v>
       </c>
       <c r="G28" s="7">
         <f>G26*(1+(G27/100))</f>
-        <v>1830.6022170142492</v>
+        <v>1509.046793200539</v>
       </c>
       <c r="H28" s="7">
         <f>H26*(1+(H27/100))</f>
-        <v>930.1194816981241</v>
+        <v>879.16401711968899</v>
       </c>
       <c r="I28" s="7">
         <f>I26*(1+(I27/100))</f>
-        <v>21923.08588695043</v>
+        <v>20530.415301241417</v>
       </c>
     </row>
   </sheetData>
@@ -5462,7 +5467,7 @@
     <row r="1" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D2" s="90" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E2" s="50" t="s">
         <v>37</v>
@@ -5474,25 +5479,25 @@
         <v>75</v>
       </c>
       <c r="H2" s="51" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I2" s="51" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J2" s="52" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D3" s="91"/>
       <c r="E3" s="53" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F3" s="54" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G3" s="92" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H3" s="93"/>
       <c r="I3" s="93"/>
@@ -5509,7 +5514,7 @@
     </row>
     <row r="5" spans="4:10" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D5" s="87" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E5" s="88"/>
       <c r="F5" s="88"/>
@@ -5520,7 +5525,7 @@
     </row>
     <row r="6" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D6" s="55" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E6" s="56">
         <v>2.6</v>
@@ -5543,7 +5548,7 @@
     </row>
     <row r="7" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D7" s="57" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E7" s="58">
         <v>0.9</v>
@@ -5566,7 +5571,7 @@
     </row>
     <row r="8" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D8" s="59" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E8" s="60">
         <v>23.4</v>
@@ -5589,7 +5594,7 @@
     </row>
     <row r="9" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D9" s="57" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E9" s="61">
         <v>105379</v>
@@ -5612,7 +5617,7 @@
     </row>
     <row r="10" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D10" s="59" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E10" s="60">
         <v>25.9</v>
@@ -5635,7 +5640,7 @@
     </row>
     <row r="11" spans="4:10" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D11" s="87" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E11" s="88"/>
       <c r="F11" s="88"/>
@@ -5646,7 +5651,7 @@
     </row>
     <row r="12" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D12" s="59" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E12" s="62">
         <v>-2072</v>
@@ -5669,7 +5674,7 @@
     </row>
     <row r="13" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D13" s="57" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E13" s="64">
         <v>-0.6</v>
@@ -5692,7 +5697,7 @@
     </row>
     <row r="14" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D14" s="59" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E14" s="62">
         <v>30980</v>
@@ -5715,7 +5720,7 @@
     </row>
     <row r="15" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D15" s="57" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E15" s="65">
         <v>53157</v>
@@ -5738,7 +5743,7 @@
     </row>
     <row r="16" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D16" s="59" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E16" s="62">
         <v>7691</v>
@@ -5761,7 +5766,7 @@
     </row>
     <row r="17" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D17" s="57" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E17" s="65">
         <v>10801</v>
@@ -5784,7 +5789,7 @@
     </row>
     <row r="18" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D18" s="59" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E18" s="62">
         <v>30251</v>
@@ -5807,7 +5812,7 @@
     </row>
     <row r="19" spans="4:10" ht="14.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D19" s="87" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E19" s="88"/>
       <c r="F19" s="88"/>
@@ -5818,7 +5823,7 @@
     </row>
     <row r="20" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D20" s="59" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E20" s="63">
         <v>8702</v>
@@ -5841,7 +5846,7 @@
     </row>
     <row r="21" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D21" s="57" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E21" s="61">
         <v>14932</v>
@@ -5864,7 +5869,7 @@
     </row>
     <row r="22" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D22" s="59" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E22" s="63">
         <v>2160</v>
@@ -5887,7 +5892,7 @@
     </row>
     <row r="23" spans="4:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="D23" s="57" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E23" s="61">
         <v>3034</v>

</xml_diff>